<commit_message>
Update realtime chat, clubs, and mobile search flows
</commit_message>
<xml_diff>
--- a/docs/import/clubs.xlsx
+++ b/docs/import/clubs.xlsx
@@ -3376,6 +3376,9 @@
       <c r="F106" t="str">
         <v>https://yandex.com/maps/2/saint-petersburg/house/Z0kYdAVgSE0HQFtjfXV4eH1iYg==/</v>
       </c>
+      <c r="I106" t="str">
+        <v>photos/1.jpeg | photos/2.jpeg | photos/3.jpeg | photos/4.jpeg | photos/5.jpeg | photos/6.jpeg</v>
+      </c>
       <c r="K106" t="str">
         <v>Беговая</v>
       </c>
@@ -3404,6 +3407,9 @@
       </c>
       <c r="F107" t="str">
         <v>https://yandex.com/maps/2/saint-petersburg/house/Z0kYdAVgSE0HQFtjfXV4eH1iYg==/</v>
+      </c>
+      <c r="I107" t="str">
+        <v>photos/1.jpeg | photos/2.jpeg | photos/3.jpeg | photos/4.jpeg | photos/5.jpeg | photos/6.jpeg</v>
       </c>
       <c r="K107" t="str">
         <v>Беговая</v>

</xml_diff>